<commit_message>
Dobrich city and Dobrichka municipality data fix.
</commit_message>
<xml_diff>
--- a/work/data/maturi_data.xlsx
+++ b/work/data/maturi_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BorisV\My Documents\dashboard\NEEBG\work\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3442A991-8CC9-4056-8DA0-AA6A177BCC79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{178FE581-40CD-410D-AEC4-E3C6FF6B89F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A348621D-5ED5-4FD9-8ED4-4EAC86F7337C}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4244" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4244" uniqueCount="280">
   <si>
     <t>Година</t>
   </si>
@@ -878,9 +878,6 @@
   <si>
     <t>2025-2026</t>
   </si>
-  <si>
-    <t>ГР.ДОБРИЧ</t>
-  </si>
 </sst>
 </file>
 
@@ -39570,7 +39567,7 @@
         <v>279</v>
       </c>
       <c r="B1917" t="s">
-        <v>280</v>
+        <v>68</v>
       </c>
       <c r="C1917">
         <v>59.204564102564099</v>
@@ -39810,7 +39807,7 @@
         <v>279</v>
       </c>
       <c r="B1929" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="C1929">
         <v>26.128620689655168</v>

</xml_diff>